<commit_message>
Corrected indexing error in rdp file
</commit_message>
<xml_diff>
--- a/data/raw/rdp.xlsx
+++ b/data/raw/rdp.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -5374,7 +5374,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -5405,14 +5405,6 @@
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -5539,7 +5531,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AV170"/>
-  <sheetFormatPr defaultColWidth="25.54296875" defaultRowHeight="14.15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="25.54296875" defaultRowHeight="14.15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.87"/>
   </cols>
@@ -5665,7 +5657,7 @@
     </row>
     <row r="2" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>39</v>
@@ -5787,7 +5779,7 @@
     </row>
     <row r="3" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>67</v>
@@ -5909,7 +5901,7 @@
     </row>
     <row r="4" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>89</v>
@@ -6031,7 +6023,7 @@
     </row>
     <row r="5" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>102</v>
@@ -6153,7 +6145,7 @@
     </row>
     <row r="6" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>102</v>
@@ -6275,7 +6267,7 @@
     </row>
     <row r="7" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>102</v>
@@ -6397,7 +6389,7 @@
     </row>
     <row r="8" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>102</v>
@@ -6519,7 +6511,7 @@
     </row>
     <row r="9" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>134</v>
@@ -6641,7 +6633,7 @@
     </row>
     <row r="10" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>145</v>
@@ -6736,7 +6728,7 @@
     </row>
     <row r="11" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>161</v>
@@ -6828,7 +6820,7 @@
     </row>
     <row r="12" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>145</v>
@@ -6956,7 +6948,7 @@
     </row>
     <row r="13" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>178</v>
@@ -7075,7 +7067,7 @@
     </row>
     <row r="14" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>178</v>
@@ -7191,7 +7183,7 @@
     </row>
     <row r="15" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>178</v>
@@ -7307,7 +7299,7 @@
     </row>
     <row r="16" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>178</v>
@@ -7426,7 +7418,7 @@
     </row>
     <row r="17" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>228</v>
@@ -7542,7 +7534,7 @@
     </row>
     <row r="18" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>228</v>
@@ -7658,7 +7650,7 @@
     </row>
     <row r="19" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>228</v>
@@ -7774,7 +7766,7 @@
     </row>
     <row r="20" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>145</v>
@@ -7896,7 +7888,7 @@
     </row>
     <row r="21" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>145</v>
@@ -8024,7 +8016,7 @@
     </row>
     <row r="22" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>161</v>
@@ -8143,7 +8135,7 @@
     </row>
     <row r="23" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>145</v>
@@ -8265,7 +8257,7 @@
     </row>
     <row r="24" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>145</v>
@@ -8387,7 +8379,7 @@
     </row>
     <row r="25" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>145</v>
@@ -8509,7 +8501,7 @@
     </row>
     <row r="26" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>145</v>
@@ -8631,7 +8623,7 @@
     </row>
     <row r="27" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B27" s="4" t="s">
         <v>145</v>
@@ -8759,7 +8751,7 @@
     </row>
     <row r="28" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B28" s="4" t="s">
         <v>145</v>
@@ -8887,7 +8879,7 @@
     </row>
     <row r="29" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>145</v>
@@ -9009,7 +9001,7 @@
     </row>
     <row r="30" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>343</v>
@@ -9131,7 +9123,7 @@
     </row>
     <row r="31" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>343</v>
@@ -9253,7 +9245,7 @@
     </row>
     <row r="32" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>360</v>
@@ -9372,7 +9364,7 @@
     </row>
     <row r="33" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B33" s="4" t="s">
         <v>370</v>
@@ -9500,7 +9492,7 @@
     </row>
     <row r="34" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>370</v>
@@ -9622,7 +9614,7 @@
     </row>
     <row r="35" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>370</v>
@@ -9744,7 +9736,7 @@
     </row>
     <row r="36" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>370</v>
@@ -9866,7 +9858,7 @@
     </row>
     <row r="37" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>370</v>
@@ -9988,7 +9980,7 @@
     </row>
     <row r="38" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B38" s="4" t="s">
         <v>370</v>
@@ -10116,7 +10108,7 @@
     </row>
     <row r="39" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>413</v>
@@ -10238,7 +10230,7 @@
     </row>
     <row r="40" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>422</v>
@@ -10360,7 +10352,7 @@
     </row>
     <row r="41" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>433</v>
@@ -10482,7 +10474,7 @@
     </row>
     <row r="42" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>433</v>
@@ -10604,7 +10596,7 @@
     </row>
     <row r="43" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>433</v>
@@ -10726,7 +10718,7 @@
     </row>
     <row r="44" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>433</v>
@@ -10848,7 +10840,7 @@
     </row>
     <row r="45" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>433</v>
@@ -10970,7 +10962,7 @@
     </row>
     <row r="46" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>466</v>
@@ -11092,7 +11084,7 @@
     </row>
     <row r="47" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="2" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>343</v>
@@ -11214,7 +11206,7 @@
     </row>
     <row r="48" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B48" s="4" t="s">
         <v>67</v>
@@ -11342,7 +11334,7 @@
     </row>
     <row r="49" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="2" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>489</v>
@@ -11464,7 +11456,7 @@
     </row>
     <row r="50" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="2" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B50" s="2" t="s">
         <v>489</v>
@@ -11586,7 +11578,7 @@
     </row>
     <row r="51" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="2" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B51" s="4" t="s">
         <v>508</v>
@@ -11714,7 +11706,7 @@
     </row>
     <row r="52" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="2" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B52" s="4" t="s">
         <v>508</v>
@@ -11842,7 +11834,7 @@
     </row>
     <row r="53" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="2" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B53" s="4" t="s">
         <v>508</v>
@@ -11970,7 +11962,7 @@
     </row>
     <row r="54" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="2" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>39</v>
@@ -12092,7 +12084,7 @@
     </row>
     <row r="55" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="2" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B55" s="2" t="s">
         <v>489</v>
@@ -12214,7 +12206,7 @@
     </row>
     <row r="56" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B56" s="2" t="s">
         <v>489</v>
@@ -12336,7 +12328,7 @@
     </row>
     <row r="57" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="2" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B57" s="2" t="s">
         <v>489</v>
@@ -12458,7 +12450,7 @@
     </row>
     <row r="58" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="2" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>489</v>
@@ -12580,7 +12572,7 @@
     </row>
     <row r="59" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="2" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B59" s="2" t="s">
         <v>581</v>
@@ -12690,7 +12682,7 @@
     </row>
     <row r="60" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="2" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B60" s="2" t="s">
         <v>489</v>
@@ -12812,7 +12804,7 @@
     </row>
     <row r="61" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="2" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B61" s="2" t="s">
         <v>601</v>
@@ -12930,8 +12922,8 @@
       </c>
     </row>
     <row r="62" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="3" t="n">
-        <v>63</v>
+      <c r="A62" s="2" t="n">
+        <v>61</v>
       </c>
       <c r="B62" s="3" t="s">
         <v>601</v>
@@ -13059,7 +13051,7 @@
     </row>
     <row r="63" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="2" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B63" s="2" t="s">
         <v>601</v>
@@ -13124,7 +13116,7 @@
     </row>
     <row r="64" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="2" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B64" s="2" t="s">
         <v>601</v>
@@ -13216,7 +13208,7 @@
     </row>
     <row r="65" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="2" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B65" s="2" t="s">
         <v>601</v>
@@ -13281,7 +13273,7 @@
     </row>
     <row r="66" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="2" t="n">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B66" s="2" t="s">
         <v>601</v>
@@ -13379,7 +13371,7 @@
     </row>
     <row r="67" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="2" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B67" s="2" t="s">
         <v>645</v>
@@ -13501,7 +13493,7 @@
     </row>
     <row r="68" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="2" t="n">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B68" s="2" t="s">
         <v>655</v>
@@ -13617,7 +13609,7 @@
     </row>
     <row r="69" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="2" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B69" s="2" t="s">
         <v>466</v>
@@ -13736,7 +13728,7 @@
     </row>
     <row r="70" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="2" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B70" s="2" t="s">
         <v>466</v>
@@ -13855,7 +13847,7 @@
     </row>
     <row r="71" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="2" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B71" s="2" t="s">
         <v>466</v>
@@ -13974,7 +13966,7 @@
     </row>
     <row r="72" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="2" t="n">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B72" s="2" t="s">
         <v>466</v>
@@ -14093,7 +14085,7 @@
     </row>
     <row r="73" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="2" t="n">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B73" s="2" t="s">
         <v>178</v>
@@ -14197,7 +14189,7 @@
     </row>
     <row r="74" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="2" t="n">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B74" s="4" t="s">
         <v>134</v>
@@ -14325,7 +14317,7 @@
     </row>
     <row r="75" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="2" t="n">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B75" s="2" t="s">
         <v>134</v>
@@ -14447,7 +14439,7 @@
     </row>
     <row r="76" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="2" t="n">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B76" s="2" t="s">
         <v>134</v>
@@ -14569,7 +14561,7 @@
     </row>
     <row r="77" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="2" t="n">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B77" s="2" t="s">
         <v>748</v>
@@ -14691,7 +14683,7 @@
     </row>
     <row r="78" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="2" t="n">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B78" s="2" t="s">
         <v>753</v>
@@ -14813,7 +14805,7 @@
     </row>
     <row r="79" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="2" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B79" s="2" t="s">
         <v>753</v>
@@ -14935,7 +14927,7 @@
     </row>
     <row r="80" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="2" t="n">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B80" s="2" t="s">
         <v>771</v>
@@ -15057,7 +15049,7 @@
     </row>
     <row r="81" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="2" t="n">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B81" s="2" t="s">
         <v>343</v>
@@ -15146,7 +15138,7 @@
     </row>
     <row r="82" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="2" t="n">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B82" s="2" t="s">
         <v>178</v>
@@ -15244,7 +15236,7 @@
     </row>
     <row r="83" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="2" t="n">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B83" s="2" t="s">
         <v>343</v>
@@ -15333,7 +15325,7 @@
     </row>
     <row r="84" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="2" t="n">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B84" s="2" t="s">
         <v>343</v>
@@ -15422,7 +15414,7 @@
     </row>
     <row r="85" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="2" t="n">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B85" s="2" t="s">
         <v>489</v>
@@ -15544,7 +15536,7 @@
     </row>
     <row r="86" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="2" t="n">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B86" s="2" t="s">
         <v>489</v>
@@ -15666,7 +15658,7 @@
     </row>
     <row r="87" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="2" t="n">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B87" s="2" t="s">
         <v>489</v>
@@ -15788,7 +15780,7 @@
     </row>
     <row r="88" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="2" t="n">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B88" s="2" t="s">
         <v>489</v>
@@ -15910,7 +15902,7 @@
     </row>
     <row r="89" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="2" t="n">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B89" s="2" t="s">
         <v>489</v>
@@ -16032,7 +16024,7 @@
     </row>
     <row r="90" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="2" t="n">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B90" s="2" t="s">
         <v>489</v>
@@ -16154,7 +16146,7 @@
     </row>
     <row r="91" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="2" t="n">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B91" s="2" t="s">
         <v>489</v>
@@ -16276,7 +16268,7 @@
     </row>
     <row r="92" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="2" t="n">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B92" s="2" t="s">
         <v>489</v>
@@ -16398,7 +16390,7 @@
     </row>
     <row r="93" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="2" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B93" s="2" t="s">
         <v>839</v>
@@ -16523,7 +16515,7 @@
     </row>
     <row r="94" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="2" t="n">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B94" s="2" t="s">
         <v>839</v>
@@ -16648,7 +16640,7 @@
     </row>
     <row r="95" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="2" t="n">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B95" s="2" t="s">
         <v>839</v>
@@ -16773,7 +16765,7 @@
     </row>
     <row r="96" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A96" s="2" t="n">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B96" s="2" t="s">
         <v>839</v>
@@ -16898,7 +16890,7 @@
     </row>
     <row r="97" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A97" s="2" t="n">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B97" s="2" t="s">
         <v>839</v>
@@ -17023,7 +17015,7 @@
     </row>
     <row r="98" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="2" t="n">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B98" s="2" t="s">
         <v>839</v>
@@ -17148,7 +17140,7 @@
     </row>
     <row r="99" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="2" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B99" s="2" t="s">
         <v>839</v>
@@ -17273,7 +17265,7 @@
     </row>
     <row r="100" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="2" t="n">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B100" s="2" t="s">
         <v>839</v>
@@ -17398,7 +17390,7 @@
     </row>
     <row r="101" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="2" t="n">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B101" s="2" t="s">
         <v>839</v>
@@ -17523,7 +17515,7 @@
     </row>
     <row r="102" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="2" t="n">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B102" s="2" t="s">
         <v>839</v>
@@ -17648,7 +17640,7 @@
     </row>
     <row r="103" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="2" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B103" s="2" t="s">
         <v>839</v>
@@ -17773,7 +17765,7 @@
     </row>
     <row r="104" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="2" t="n">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="B104" s="2" t="s">
         <v>422</v>
@@ -17898,7 +17890,7 @@
     </row>
     <row r="105" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A105" s="2" t="n">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="B105" s="2" t="s">
         <v>422</v>
@@ -18023,7 +18015,7 @@
     </row>
     <row r="106" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A106" s="2" t="n">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="B106" s="2" t="s">
         <v>422</v>
@@ -18148,7 +18140,7 @@
     </row>
     <row r="107" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A107" s="2" t="n">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="B107" s="2" t="s">
         <v>422</v>
@@ -18273,7 +18265,7 @@
     </row>
     <row r="108" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A108" s="2" t="n">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="B108" s="2" t="s">
         <v>422</v>
@@ -18398,7 +18390,7 @@
     </row>
     <row r="109" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A109" s="2" t="n">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="B109" s="2" t="s">
         <v>422</v>
@@ -18523,7 +18515,7 @@
     </row>
     <row r="110" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="2" t="n">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="B110" s="2" t="s">
         <v>422</v>
@@ -18648,7 +18640,7 @@
     </row>
     <row r="111" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A111" s="2" t="n">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="B111" s="2" t="s">
         <v>422</v>
@@ -18773,7 +18765,7 @@
     </row>
     <row r="112" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A112" s="2" t="n">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="B112" s="2" t="s">
         <v>422</v>
@@ -18898,7 +18890,7 @@
     </row>
     <row r="113" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A113" s="2" t="n">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="B113" s="2" t="s">
         <v>422</v>
@@ -19023,7 +19015,7 @@
     </row>
     <row r="114" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A114" s="2" t="n">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="B114" s="2" t="s">
         <v>422</v>
@@ -19148,7 +19140,7 @@
     </row>
     <row r="115" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A115" s="2" t="n">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="B115" s="2" t="s">
         <v>422</v>
@@ -19273,7 +19265,7 @@
     </row>
     <row r="116" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A116" s="2" t="n">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="B116" s="2" t="s">
         <v>422</v>
@@ -19398,7 +19390,7 @@
     </row>
     <row r="117" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A117" s="2" t="n">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="B117" s="2" t="s">
         <v>422</v>
@@ -19523,7 +19515,7 @@
     </row>
     <row r="118" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A118" s="2" t="n">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="B118" s="2" t="s">
         <v>422</v>
@@ -19648,7 +19640,7 @@
     </row>
     <row r="119" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A119" s="2" t="n">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="B119" s="2" t="s">
         <v>89</v>
@@ -19770,7 +19762,7 @@
     </row>
     <row r="120" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A120" s="2" t="n">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="B120" s="2" t="s">
         <v>89</v>
@@ -19892,7 +19884,7 @@
     </row>
     <row r="121" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A121" s="2" t="n">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="B121" s="2" t="s">
         <v>89</v>
@@ -20014,7 +20006,7 @@
     </row>
     <row r="122" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A122" s="2" t="n">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="B122" s="2" t="s">
         <v>89</v>
@@ -20136,7 +20128,7 @@
     </row>
     <row r="123" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A123" s="2" t="n">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="B123" s="2" t="s">
         <v>89</v>
@@ -20258,7 +20250,7 @@
     </row>
     <row r="124" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A124" s="2" t="n">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="B124" s="2" t="s">
         <v>89</v>
@@ -20380,7 +20372,7 @@
     </row>
     <row r="125" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A125" s="2" t="n">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="B125" s="2" t="s">
         <v>178</v>
@@ -20502,7 +20494,7 @@
     </row>
     <row r="126" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A126" s="2" t="n">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="B126" s="2" t="s">
         <v>178</v>
@@ -20624,7 +20616,7 @@
     </row>
     <row r="127" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A127" s="2" t="n">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="B127" s="2" t="s">
         <v>178</v>
@@ -20746,7 +20738,7 @@
     </row>
     <row r="128" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A128" s="2" t="n">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="B128" s="4" t="s">
         <v>178</v>
@@ -20874,7 +20866,7 @@
     </row>
     <row r="129" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A129" s="2" t="n">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="B129" s="2" t="s">
         <v>178</v>
@@ -20996,7 +20988,7 @@
     </row>
     <row r="130" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A130" s="2" t="n">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="B130" s="2" t="s">
         <v>178</v>
@@ -21118,7 +21110,7 @@
     </row>
     <row r="131" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A131" s="2" t="n">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="B131" s="2" t="s">
         <v>178</v>
@@ -21240,7 +21232,7 @@
     </row>
     <row r="132" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A132" s="2" t="n">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="B132" s="2" t="s">
         <v>987</v>
@@ -21362,7 +21354,7 @@
     </row>
     <row r="133" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A133" s="2" t="n">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="B133" s="2" t="s">
         <v>508</v>
@@ -21484,7 +21476,7 @@
     </row>
     <row r="134" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A134" s="2" t="n">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="B134" s="2" t="s">
         <v>466</v>
@@ -21603,7 +21595,7 @@
     </row>
     <row r="135" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A135" s="2" t="n">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="B135" s="2" t="s">
         <v>987</v>
@@ -21725,7 +21717,7 @@
     </row>
     <row r="136" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A136" s="2" t="n">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="B136" s="2" t="s">
         <v>987</v>
@@ -21847,7 +21839,7 @@
     </row>
     <row r="137" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A137" s="2" t="n">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="B137" s="2" t="s">
         <v>178</v>
@@ -21969,7 +21961,7 @@
     </row>
     <row r="138" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A138" s="2" t="n">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="B138" s="2" t="s">
         <v>466</v>
@@ -22091,7 +22083,7 @@
     </row>
     <row r="139" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A139" s="2" t="n">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="B139" s="2" t="s">
         <v>1045</v>
@@ -22213,7 +22205,7 @@
     </row>
     <row r="140" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A140" s="2" t="n">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="B140" s="2" t="s">
         <v>987</v>
@@ -22335,7 +22327,7 @@
     </row>
     <row r="141" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A141" s="2" t="n">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="B141" s="2" t="s">
         <v>466</v>
@@ -22454,7 +22446,7 @@
     </row>
     <row r="142" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A142" s="2" t="n">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="B142" s="2" t="s">
         <v>987</v>
@@ -22576,7 +22568,7 @@
     </row>
     <row r="143" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A143" s="2" t="n">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="B143" s="2" t="s">
         <v>987</v>
@@ -22698,7 +22690,7 @@
     </row>
     <row r="144" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A144" s="2" t="n">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="B144" s="2" t="s">
         <v>987</v>
@@ -22820,7 +22812,7 @@
     </row>
     <row r="145" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A145" s="2" t="n">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="B145" s="2" t="s">
         <v>1045</v>
@@ -22942,7 +22934,7 @@
     </row>
     <row r="146" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A146" s="2" t="n">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="B146" s="2" t="s">
         <v>466</v>
@@ -23061,7 +23053,7 @@
     </row>
     <row r="147" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A147" s="2" t="n">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="B147" s="2" t="s">
         <v>466</v>
@@ -23180,7 +23172,7 @@
     </row>
     <row r="148" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A148" s="2" t="n">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="B148" s="2" t="s">
         <v>1073</v>
@@ -23302,7 +23294,7 @@
     </row>
     <row r="149" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A149" s="2" t="n">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="B149" s="2" t="s">
         <v>1073</v>
@@ -23424,7 +23416,7 @@
     </row>
     <row r="150" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A150" s="2" t="n">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="B150" s="2" t="s">
         <v>1045</v>
@@ -23546,7 +23538,7 @@
     </row>
     <row r="151" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A151" s="2" t="n">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="B151" s="2" t="s">
         <v>1045</v>
@@ -23668,7 +23660,7 @@
     </row>
     <row r="152" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A152" s="2" t="n">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="B152" s="2" t="s">
         <v>1086</v>
@@ -23790,7 +23782,7 @@
     </row>
     <row r="153" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A153" s="2" t="n">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="B153" s="2" t="s">
         <v>1045</v>
@@ -23912,7 +23904,7 @@
     </row>
     <row r="154" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A154" s="2" t="n">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="B154" s="2" t="s">
         <v>1097</v>
@@ -24034,7 +24026,7 @@
     </row>
     <row r="155" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A155" s="2" t="n">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="B155" s="2" t="s">
         <v>1073</v>
@@ -24156,7 +24148,7 @@
     </row>
     <row r="156" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A156" s="2" t="n">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="B156" s="2" t="s">
         <v>645</v>
@@ -24275,7 +24267,7 @@
     </row>
     <row r="157" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A157" s="2" t="n">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="B157" s="2" t="s">
         <v>753</v>
@@ -24397,7 +24389,7 @@
     </row>
     <row r="158" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A158" s="2" t="n">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B158" s="2" t="s">
         <v>753</v>
@@ -24519,7 +24511,7 @@
     </row>
     <row r="159" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A159" s="2" t="n">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="B159" s="2" t="s">
         <v>753</v>
@@ -24641,7 +24633,7 @@
     </row>
     <row r="160" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A160" s="2" t="n">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="B160" s="2" t="s">
         <v>753</v>
@@ -24763,7 +24755,7 @@
     </row>
     <row r="161" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A161" s="2" t="n">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="B161" s="2" t="s">
         <v>753</v>
@@ -24885,7 +24877,7 @@
     </row>
     <row r="162" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A162" s="2" t="n">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="B162" s="2" t="s">
         <v>753</v>
@@ -25007,7 +24999,7 @@
     </row>
     <row r="163" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A163" s="2" t="n">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="B163" s="2" t="s">
         <v>753</v>
@@ -25129,7 +25121,7 @@
     </row>
     <row r="164" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A164" s="2" t="n">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="B164" s="2" t="s">
         <v>645</v>
@@ -25251,7 +25243,7 @@
     </row>
     <row r="165" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A165" s="2" t="n">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="B165" s="3" t="s">
         <v>178</v>
@@ -25379,7 +25371,7 @@
     </row>
     <row r="166" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A166" s="2" t="n">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="B166" s="3" t="s">
         <v>1166</v>
@@ -25507,7 +25499,7 @@
     </row>
     <row r="167" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A167" s="2" t="n">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="B167" s="3" t="s">
         <v>1166</v>
@@ -25635,7 +25627,7 @@
     </row>
     <row r="168" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A168" s="2" t="n">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="B168" s="3" t="s">
         <v>178</v>
@@ -25763,7 +25755,7 @@
     </row>
     <row r="169" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A169" s="2" t="n">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="B169" s="3" t="s">
         <v>1217</v>
@@ -25891,131 +25883,131 @@
     </row>
     <row r="170" customFormat="false" ht="14.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A170" s="2" t="n">
-        <v>176</v>
-      </c>
-      <c r="B170" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="B170" s="3" t="s">
         <v>1217</v>
       </c>
-      <c r="C170" s="8" t="s">
+      <c r="C170" s="3" t="s">
         <v>1218</v>
       </c>
-      <c r="D170" s="8" t="s">
+      <c r="D170" s="3" t="s">
         <v>1233</v>
       </c>
-      <c r="E170" s="8" t="s">
+      <c r="E170" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="F170" s="8" t="s">
+      <c r="F170" s="3" t="s">
         <v>1234</v>
       </c>
-      <c r="G170" s="8" t="s">
+      <c r="G170" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="H170" s="8" t="s">
+      <c r="H170" s="3" t="s">
         <v>1234</v>
       </c>
-      <c r="I170" s="8" t="s">
+      <c r="I170" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="J170" s="8" t="s">
+      <c r="J170" s="3" t="s">
         <v>1234</v>
       </c>
-      <c r="K170" s="8" t="s">
+      <c r="K170" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="L170" s="8" t="s">
+      <c r="L170" s="3" t="s">
         <v>1234</v>
       </c>
-      <c r="M170" s="8" t="s">
+      <c r="M170" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="N170" s="8" t="s">
+      <c r="N170" s="3" t="s">
         <v>1235</v>
       </c>
-      <c r="O170" s="8" t="s">
+      <c r="O170" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="P170" s="8" t="s">
+      <c r="P170" s="3" t="s">
         <v>1235</v>
       </c>
-      <c r="Q170" s="8" t="s">
+      <c r="Q170" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="R170" s="8" t="s">
+      <c r="R170" s="3" t="s">
         <v>1235</v>
       </c>
-      <c r="S170" s="8" t="s">
+      <c r="S170" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="T170" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="U170" s="8" t="s">
+      <c r="T170" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="U170" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="V170" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="W170" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="X170" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="Y170" s="8" t="s">
+      <c r="V170" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="W170" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="X170" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="Y170" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="Z170" s="8" t="s">
+      <c r="Z170" s="3" t="s">
         <v>1236</v>
       </c>
-      <c r="AA170" s="8" t="s">
+      <c r="AA170" s="3" t="s">
         <v>301</v>
       </c>
-      <c r="AB170" s="8" t="s">
+      <c r="AB170" s="3" t="s">
         <v>1237</v>
       </c>
-      <c r="AC170" s="8" t="s">
+      <c r="AC170" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="AD170" s="8" t="s">
+      <c r="AD170" s="3" t="s">
         <v>1237</v>
       </c>
-      <c r="AE170" s="8" t="s">
+      <c r="AE170" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="AF170" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="AG170" s="8" t="s">
+      <c r="AF170" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="AG170" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="AH170" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="AI170" s="8" t="s">
+      <c r="AH170" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="AI170" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="AJ170" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="AK170" s="8" t="s">
+      <c r="AJ170" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="AK170" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="AL170" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="AM170" s="8" t="s">
+      <c r="AL170" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="AM170" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="AN170" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="AO170" s="9"/>
-      <c r="AR170" s="9"/>
-      <c r="AS170" s="9"/>
-      <c r="AT170" s="9"/>
-      <c r="AU170" s="9"/>
-      <c r="AV170" s="9"/>
+      <c r="AN170" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="AO170" s="2"/>
+      <c r="AR170" s="2"/>
+      <c r="AS170" s="2"/>
+      <c r="AT170" s="2"/>
+      <c r="AU170" s="2"/>
+      <c r="AV170" s="2"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>